<commit_message>
Scrub internal IPs from the dev sanity test spreadsheet
* Replace internal infrastructure IP addresses in the vios_dev_sanity test steps with placeholders.

Signed-off-by: Divy Sitlani <dsitlani@nvidia.com>
</commit_message>
<xml_diff>
--- a/services/vios/test/vios_dev_sanity.xlsx
+++ b/services/vios/test/vios_dev_sanity.xlsx
@@ -1060,7 +1060,7 @@
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>1. Get valid RTSP streams by calling REST API GET: http://10.24.216.253:31000/api/v1/sensor/streams
+          <t>1. Get valid RTSP streams by calling REST API GET: http://&lt;HOST&gt;:31000/api/v1/sensor/streams
 2. Open http://ip:30888/vst/#/sensor-management
 3. Look for Add new sensors component. Ensure RTSP URL is toggled on.
 4. Enter RTSP URL in URL section.
@@ -1169,7 +1169,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Open http://10.41.26.58:31000/#/media-upload for nvstreamer file upload page.
+          <t xml:space="preserve">1. Open http://&lt;HOST&gt;:31000/#/media-upload for nvstreamer file upload page.
 2. Look for "Upload files" section. It has area that can be clicked to select files to upload or we can drag and drop files there to upload.
 3. Scan current directory to look for .mkv or .mp4 files. Use those files to upload in Nvstreamer.
 4. Files to upload can generally be found in test/bdd_tests/data or tools/data directories. If not found there scan in other places. 
@@ -1274,7 +1274,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Table populated: 10 rows, columns Name/RTSP URL/Type/Resolution. RTSP URL format rtsp://10.41.26.58:30XXX/live/&lt;sensor_name&gt; confirmed valid. Resolution values: 1920x1080 and 1280x720.</t>
+          <t>Table populated: 10 rows, columns Name/RTSP URL/Type/Resolution. RTSP URL format rtsp://&lt;HOST&gt;:30XXX/live/&lt;sensor_name&gt; confirmed valid. Resolution values: 1920x1080 and 1280x720.</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Expand VIOS dev sanity suite and harden test isolation
- Add 10 sanity tests: direct file upload, clip export/download, media
  delete, record settings, live/replay snapshot, file-type sensor delete,
  and regression guards for dropdown filtering, H265 codec, and audio track
- Replace hardcoded IPs/hosts with placeholders; source RTSP and H265
  streams from the local NvStreamer
- Add a startup environment preflight that resolves URLs and image tags
  from the live environment and prompts for a NvStreamer IP only when none
  can be detected locally
- Add run-start baseline cleanup and mandatory per-test teardown so the
  suite is idempotent and free of false negatives from leftover state
- Select only online sensors for stream and video-wall tests

Signed-off-by: Prakhar Shukla <prakhars@nvidia.com>
</commit_message>
<xml_diff>
--- a/services/vios/test/vios_dev_sanity.xlsx
+++ b/services/vios/test/vios_dev_sanity.xlsx
@@ -836,7 +836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.7109375" customWidth="1" min="1" max="1"/>
@@ -890,16 +890,8 @@
           <t>Live WebRTC Stream</t>
         </is>
       </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="D2" s="16" t="inlineStr">
-        <is>
-          <t>PeerConnectionManager::checkStreamSanity returns 'Streaming not yet started' for all sensors. RTSP streams confirmed active via ffprobe. JS dispatch (mousedown+click) opened dropdown correctly; visibleAcs[1] = Select Sensors confirmed. Backend live WebRTC state not initialized — not a UI selector issue.</t>
-        </is>
-      </c>
+      <c r="C2" s="17" t="n"/>
+      <c r="D2" s="16" t="n"/>
       <c r="E2" s="16" t="inlineStr">
         <is>
           <t>VIOS deployment should be up and healthy. Atleast one stream should be present in system.</t>
@@ -927,16 +919,8 @@
           <t>Replay WebRTC Stream</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>nvidia_10sec replay: videoWidth=1920, videoHeight=1080, readyState=4, paused=false, currentTime 28.37-&gt;40.50 in 5s. Timeline 11:27:10-16:08:15. Speed controls visible. JS dispatch visibleAcs[1]=Select Sensors confirmed working.</t>
-        </is>
-      </c>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="inlineStr">
         <is>
           <t>VIOS deployment should be up and healthy. Atleast one stream should be present in system.</t>
@@ -964,19 +948,11 @@
           <t>Video Wall WebRTC Steam</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>3 sensors selected; body shows 'Streaming 3 sensors'; 1 active video (videoWidth=1920, readyState=4, currentTime=201.6); Stop button enabled. Confirmed: exactly 1 visible AC on video-wall (visibleAcs[0]); compositor produces 1 merged WebRTC stream (1 video element with videoWidth&gt;0).</t>
-        </is>
-      </c>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="3" t="n"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>VIOS deployment should be up and healthy. Atleast two streams should be present in system.</t>
+          <t>VIOS deployment should be up and healthy. Atleast two streams should be present in system. Select only ONLINE sensors for the video wall - never offline/removed entries (an offline orphan from a prior test will fail playback for reasons unrelated to the product). The environment should be at a clean baseline (see the run's baseline-cleanup step).</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
@@ -1002,25 +978,17 @@
           <t>UI Dashboard stats, tables and info</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>15 total sensors, 0 offline, 0 bad state, 0 gaps, 15 recording. 'All services available' shown. Timeline section present. All stat cards populated.</t>
-        </is>
-      </c>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>VIOS deployment should be up and healthy. Atleast one stream should be present in system.</t>
+          <t>VIOS deployment should be up and healthy. Atleast one stream should be present in system. The environment must be at a clean baseline before this test: orphaned/offline sensors left over from earlier tests are test artifacts, not product defects, and must be cleaned up first (see the run's baseline-cleanup step). The Offline/Bad-state/Gaps assertions are judged against the cleaned baseline set of online streams.</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
           <t>1. Goto http://ip:30888/vst/#/dashboard
-2. The dashboard should not successfully.
+2. The dashboard should load successfully.
 3. The dashboard should show "All services available"
 4. Total sensors are shown in widget "Total sensors"
 5. The recordings should not have any recording gaps. Look for "Sensors with recording gaps" widget.
@@ -1043,16 +1011,8 @@
           <t>Adding sensor using RTSP stream</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Sensor sanity_test_rtsp added (UUID 3324b17f). Dashboard count: 15-&gt;16. CRITICAL: standard input.value=x fails to enable Add Sensor button; must use native HTMLInputElement.prototype value setter + dispatchEvent('input','change') to trigger React state.</t>
-        </is>
-      </c>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="3" t="n"/>
       <c r="E6" s="3" t="inlineStr">
         <is>
           <t>VIOS deployment should be up and healthy.</t>
@@ -1060,15 +1020,17 @@
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>1. Get valid RTSP streams by calling REST API GET: http://&lt;HOST&gt;:31000/api/v1/sensor/streams
+          <t>1. Get valid RTSP streams by calling REST API GET: http://localhost:31000/api/v1/sensor/streams (the local NvStreamer). Use the resolved NvStreamer host/port from the run's environment preflight if it is not localhost:31000.
+   NOTE: VIOS auto-imports the local NvStreamer streams, and it deduplicates by stream identity - re-adding a stream that already exists returns HTTP 400 'Sensor exists already', which is correct product behavior, not a failure. To exercise the add path cleanly, pick a stream that is NOT already present in GET http://ip:30888/vst/api/v1/sensor/streams; if every NvStreamer stream is already imported, temporarily remove one baseline sensor and re-add it by its RTSP URL, then restore it.
 2. Open http://ip:30888/vst/#/sensor-management
 3. Look for Add new sensors component. Ensure RTSP URL is toggled on.
-4. Enter RTSP URL in URL section.
-5. Enter name in name section. If RTSP URL is "rtsp://ip:31554/path/name.mp4" then use name as "name.mp4".
-6. Submit by clicking on "Add sensor" button.
-7. Now open dashboard "http://ip:30888/vst/#/dashboard and check if that sensor is present, has no errors and is recording.
-8. You can also check it by calling REST API GET: "http://ip:30888/vst/api/v1/sensor/streams". Ideally we should check both by Dashboard and by calling REST API.
-9. Add another RTSP URL, but this time don't give name. The VIOS should automatically assign unqiue name to sensors like sensor_1, sensor_2 etc. Confirm it by adding two RTSP streams without giving names.</t>
+4. Enter the RTSP URL in the URL section.
+5. Enter a UNIQUE, run-scoped name (e.g. sanity_rtsp_&lt;HHMMSS&gt;) so it cannot collide with existing sensors. (If the RTSP URL is rtsp://ip:31554/path/name.mp4 a name like name.mp4 is also acceptable as long as it is unique.)
+6. Submit by clicking on "Add sensor".
+7. Open dashboard http://ip:30888/vst/#/dashboard and check the sensor is present, has no errors and is recording.
+8. Also verify via REST API GET: http://ip:30888/vst/api/v1/sensor/streams. Ideally check both Dashboard and REST API.
+9. Auto-naming check: add two more RTSP streams WITHOUT giving a name (use distinct, not-already-imported URLs). VIOS should auto-assign unique names like sensor_1, sensor_2. Confirm both are created with unique names.
+10. CLEANUP (mandatory, even if an earlier step failed): remove EVERY sensor this test added (the named one and the two auto-named ones) via the Remove Sensors UI or DELETE REST API, and confirm the sensor count returns to the pre-test baseline. The test must leave the system exactly as it found it.</t>
         </is>
       </c>
     </row>
@@ -1083,16 +1045,8 @@
           <t>Removing senor</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>sanity_test_rtsp removed; dashboard returns to 15 sensors; API confirms state='removed'. Note: button label is 'Remove Sensor' (singular) not 'Remove Sensors' as shown in UI selector docs.</t>
-        </is>
-      </c>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>VIOS deployment should be up and healthy. Atleast one stream should be present in system.</t>
@@ -1120,16 +1074,8 @@
           <t>Adding sensor using IP address and password</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Test steps say 'SKIP this test until further update.'</t>
-        </is>
-      </c>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="inlineStr">
         <is>
           <t>VIOS deployment should be up and healthy.</t>
@@ -1152,16 +1098,8 @@
           <t>Scaning new sensors to VIOS that are added to NvStreamer at runtime</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Scan for Sensors clicked; API count 15-&gt;16 after scan; dashboard confirms 16 total sensors. New NvStreamer-registered stream picked up.</t>
-        </is>
-      </c>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="5" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>VIOS and NvStreamer deployment should be up and healthy.</t>
@@ -1169,7 +1107,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Open http://&lt;HOST&gt;:31000/#/media-upload for nvstreamer file upload page.
+          <t>1. Open http://ip:31000/#/media-upload for nvstreamer file upload page.
 2. Look for "Upload files" section. It has area that can be clicked to select files to upload or we can drag and drop files there to upload.
 3. Scan current directory to look for .mkv or .mp4 files. Use those files to upload in Nvstreamer.
 4. Files to upload can generally be found in test/bdd_tests/data or tools/data directories. If not found there scan in other places. 
@@ -1180,7 +1118,7 @@
 9. Look for "Scan Sensors" component and click on "Scan for sensors" button.
 10. Now open VIOS dashboard http://ip:30888/vst/#/dashboard, the new sensor that we added in nvstreamer should be picked up by VIOS after scan. It should come up in dashboard.
 11. You can also check it by calling REST API GET: "http://ip:30888/vst/api/v1/sensor/streams". Ideally we should check both by Dashboard and by calling REST API.
-</t>
+12. CLEANUP (mandatory, even if an earlier step failed): remove the test sensor that was picked up by the scan via the Remove Sensors UI or DELETE REST API, and delete the file uploaded to NvStreamer if possible. Confirm the VIOS sensor count returns to the pre-test baseline so no orphaned/duplicate sensors are left behind for later runs.</t>
         </is>
       </c>
     </row>
@@ -1195,16 +1133,8 @@
           <t>Sensor configuration like image and encode settings. Only applicable for ONVIF sensors.</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Test steps say 'SKIP this test until further update.' (Only applicable for ONVIF sensors; none present.)</t>
-        </is>
-      </c>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="3" t="n"/>
       <c r="E10" s="3" t="inlineStr">
         <is>
           <t>VIOS deployment should be up and healthy. Atleast one ONVIF stream should be present in system.</t>
@@ -1227,16 +1157,8 @@
           <t>Sensor details like name, tags, sensor position etc. Network information is applicable only for ONVIF sensors.</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>nvidia_10sec selected; Name='nvidia_10sec', SensorID='nvidia_10sec', state=online (API confirmed). Network info unavailable — expected for RTSP/NvStreamer sensors (non-ONVIF). JS dispatch on visibleAcs[0]=Select Sensor worked correctly (1 visible AC on sensor-details page).</t>
-        </is>
-      </c>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>VIOS deployment should be up and healthy. Atleast one stream should be present in system.</t>
@@ -1267,16 +1189,8 @@
 The RTSP URL will not be valid if it’s a file type sensor. RTSP URL is valid only if RTSP stream was added to VST or ONVIF sensor added using IP address. If file was uploaded to VST to create sensor then for it RTSP URL will be a file path and it will not be valid.</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Table populated: 10 rows, columns Name/RTSP URL/Type/Resolution. RTSP URL format rtsp://&lt;HOST&gt;:30XXX/live/&lt;sensor_name&gt; confirmed valid. Resolution values: 1920x1080 and 1280x720.</t>
-        </is>
-      </c>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="7" t="n"/>
       <c r="E12" s="7" t="inlineStr">
         <is>
           <t>VIOS deployment should be up and healthy. Atleast one stream should be present in system.</t>
@@ -1287,6 +1201,292 @@
           <t>1. Goto http://ip:30888/vst/#/stream-details
 2. You should see a table with colmunns Name, RTSP URL,	Type and Resolution
 3. The table should list all sensors. All RTSP streams should have valid RTSP streams and resolutions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="110" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>File Upload</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Uploading a video file directly to VIOS using PUT File Upload</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="n"/>
+      <c r="D13" s="16" t="n"/>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>VIOS deployment should be up and healthy.</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>1. Goto http://ip:30888/vst/#/media-management
+2. Look for the "Upload Parameters" / "PUT File Upload" section.
+3. Scan current directory for .mkv or .mp4 files. Files can generally be found in test/bdd_tests/data or tools/data. If not there, scan other places.
+4. Optionally set Custom Filename, Sensor ID and Timestamp. Toggle Transcode / multi-part upload as needed.
+5. Upload the file using the "Click or drag a file to upload" area and click "PUT File Upload".
+6. After upload, open http://ip:30888/vst/#/dashboard and confirm the new sensor is present, has no errors and is recording.
+7. Also verify via REST API GET: http://ip:30888/vst/api/v1/sensor/streams that the uploaded sensor exists. Ideally check both Dashboard and REST API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="110" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Media Management</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Video clip export and download using Media URL Generator</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="16" t="n"/>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>VIOS deployment should be up and healthy. At least one stream with recordings should be present.</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>1. Goto http://ip:30888/vst/#/media-management
+2. In the "Media URL Generator" section, select a sensor that has recordings.
+3. Set Start Time and End Time (ISO 8601) within the recorded timeline, choose Container Format (mp4 or ts), optionally Enable Audio and set Expiry Minutes.
+4. Click "Generate Video URL".
+5. Click "Download Video" (or use "Copy Download URL" and GET it via curl) and confirm a valid, non-empty video file is downloaded.
+6. Optionally validate the downloaded clip with ffprobe (correct duration, codec, resolution).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="110" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Media Management</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Deleting a media/video entry from Media Streams</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>VIOS deployment should be up and healthy. At least one recorded media entry should be present.</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>1. Goto http://ip:30888/vst/#/media-management
+2. In the "Media Streams" section, locate an existing video entry.
+3. Click "Delete Video" for that entry.
+4. Confirm the entry is removed from the Media Streams list.
+5. Verify via REST API that the corresponding recording/file is no longer returned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="110" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Sensor Management</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Deleting a file-type sensor removes it completely (no stale entry). Guards against Bug 6217837.</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>VIOS deployment should be up and healthy.</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>1. Create a file-type sensor by uploading a file (via Media Management PUT upload, or NvStreamer file upload followed by Scan for sensors).
+2. Confirm the sensor in dashboard http://ip:30888/vst/#/dashboard and via REST API GET http://ip:30888/vst/api/v1/sensor/streams
+3. Open http://ip:30888/vst/#/sensor-management and remove that file-type sensor using the "Remove Sensors" component.
+4. Reload the dashboard and confirm the sensor is fully gone - not present and no stale or blank-named entry remains.
+5. Verify via REST API GET http://ip:30888/vst/api/v1/sensor/streams that the sensor is removed, and confirm it no longer appears in the dropdowns on sensor-details and stream-details pages.
+6. This test guards against Bug 6217837 where file-type sensors remained visible in the UI after deletion (delete only removed VST storage, not the sensor entry).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="110" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Sensor Management</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>UI dropdowns exclude removed and blank-named sensors. Guards against Bug 6150793.</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>VIOS deployment should be up and healthy. At least one stream should be present.</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>1. Call REST API GET http://ip:30888/vst/api/v1/sensor/list and note any entries with state='removed' or an empty name.
+2. Open http://ip:30888/vst/#/sensor-details and http://ip:30888/vst/#/live-streams
+3. Open each "Select Sensor(s)" dropdown.
+4. Confirm that no blank-named entries appear and no sensors with state='removed' are listed in any dropdown.
+5. This test guards against Bug 6150793 where removed and blank-named sensor entries leaked into UI dropdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="110" customHeight="1">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Sensor Management</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Adding a sensor with an invalid RTSP URL shows an error and creates no sensor (negative test)</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>VIOS deployment should be up and healthy.</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>1. Open http://ip:30888/vst/#/sensor-management
+2. In the "Add new sensors" component, ensure RTSP URL is toggled on.
+3. Enter an invalid RTSP URL (e.g. rtsp://invalid-host:554/does-not-exist) and a name.
+4. Click "Add sensor".
+5. Confirm an appropriate error is shown and the sensor is NOT added. Verify the dashboard sensor count is unchanged and that the sensor is absent from REST API GET http://ip:30888/vst/api/v1/sensor/streams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="110" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Record Settings</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Changing a sensor's recording status / schedule</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>VIOS deployment should be up and healthy. At least one stream should be present.</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>1. Goto http://ip:30888/vst/#/record-settings
+2. Select a sensor. Use "Change Status" to toggle recording Off and then On (or set a recording schedule window using Start Time / End Time with Day/Hour/Minute).
+3. Click "Submit".
+4. Open http://ip:30888/vst/#/dashboard and confirm the sensor's recording state reflects the change.
+5. Restore the original recording status afterwards so other tests are unaffected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="110" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Live and replay image (snapshot) capture</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>VIOS deployment should be up and healthy. At least one stream with recordings should be present.</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>1. Goto http://ip:30888/vst/#/media-management (image/snapshot controls are also available on the Experimental page).
+2. Select a sensor. Click "Get Live Image URL", then open or GET the returned URL and confirm a valid, non-empty JPEG is returned.
+3. For replay, set a Replay Start Time within the recorded timeline, click "Get Replay Image URL", GET the returned URL and confirm a valid JPEG is returned.
+4. Both the live and replay snapshots should return non-empty, valid images.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="110" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Stream Details</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Manually-added H265 RTSP stream reports correct Type (H265) and metadata. Guards against Bug 6169252.</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>VIOS deployment should be up and healthy. A valid H265 RTSP stream should be available.</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>1. Get a valid H265 RTSP stream URL by calling REST API GET: http://localhost:31000/api/v1/sensor/streams (the local NvStreamer; use the resolved NvStreamer host/port from the run's environment preflight if not localhost:31000). Pick a stream whose codec is H265, e.g. sample_10sec_h265 or Building_K_Cam1_2min_h265.
+2. Open http://ip:30888/vst/#/sensor-management and add the H265 RTSP stream via the "Add new sensors" component (RTSP URL toggled on). Use a unique run-scoped name.
+3. Goto http://ip:30888/vst/#/stream-details
+4. Locate the newly added sensor row. Confirm the Type column shows H265 (not H264) and that Resolution and other metadata are populated correctly.
+5. Also verify via REST API GET http://ip:30888/vst/api/v1/sensor/streams that the codec/type is reported as H265 with complete metadata.
+6. This test guards against Bug 6169252 where manually-added H265 RTSP streams were reported as H264 with missing metadata.
+7. CLEANUP (mandatory): remove the H265 sensor added by this test so the system returns to its pre-test baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="110" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Recorded Streams</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Recorded / republished stream contains an audio track. Guards against Bug 6201789.</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>VIOS deployment should be up and healthy. A stream with audio (e.g. audio_video) should be present.</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>1. Identify a sensor that has an audio track (e.g. the audio_video stream).
+2. Goto http://ip:30888/vst/#/media-management and use the Media URL Generator to export a clip for that sensor with "Enable Audio" turned on (or download a recorded clip).
+3. Download the clip via "Download Video".
+4. Inspect the downloaded clip with ffprobe and confirm an audio stream is present alongside the video stream.
+5. Optionally also confirm audio on the republished RTSP stream (rtsp://ip:30XXX/live/&lt;sensor_name&gt;) using ffprobe.
+6. This test guards against Bug 6201789 where NvStreamer-republished RTSP streams did not include the audio track.</t>
         </is>
       </c>
     </row>

</xml_diff>